<commit_message>
Raise gross investment return assumption to 11%
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NuskepMCVmLKKsfCHMW5fw
</commit_message>
<xml_diff>
--- a/outputs/Buy_vs_Rent_Cape_Town.xlsx
+++ b/outputs/Buy_vs_Rent_Cape_Town.xlsx
@@ -219,7 +219,7 @@
     <t xml:space="preserve">Investment return, gross (p.a., nominal)</t>
   </si>
   <si>
-    <t xml:space="preserve">Conservative for a growth/equity-heavy portfolio: ~CPI 4.5% + 5.5% real.</t>
+    <t xml:space="preserve">User-chosen conservative equity return: ~CPI 4.5% + 6.5% real.</t>
   </si>
   <si>
     <t xml:space="preserve">Fund / platform fees (p.a.)</t>
@@ -976,37 +976,37 @@
                   <c:v>5962145.93244849</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>6582631.39844278</c:v>
+                  <c:v>6582647.52498468</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>7272376.66912875</c:v>
+                  <c:v>7272528.46908091</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8038203.58167651</c:v>
+                  <c:v>8038808.51459033</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>8887599.9585631</c:v>
+                  <c:v>8889215.50285084</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9828784.8360684</c:v>
+                  <c:v>9832256.78469764</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>10870780.1541459</c:v>
+                  <c:v>10877297.8684327</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>11889560.2077326</c:v>
+                  <c:v>11902153.4038142</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>12997970.6788673</c:v>
+                  <c:v>13021938.2388558</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>14203647.2672151</c:v>
+                  <c:v>14245373.6057881</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>15514859.4303046</c:v>
+                  <c:v>15581972.2295863</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>16940561.9261636</c:v>
+                  <c:v>17042109.367774</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1162,79 +1162,79 @@
                   <c:v>848394</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1105101.0744721</c:v>
+                  <c:v>1112831.22078536</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1369038.8542117</c:v>
+                  <c:v>1387354.81953521</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1640332.79926112</c:v>
+                  <c:v>1672429.1817303</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1919093.54192227</c:v>
+                  <c:v>1968535.82501265</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2205414.37860174</c:v>
+                  <c:v>2276173.60499552</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2499368.49400676</c:v>
+                  <c:v>2595858.86993307</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2801005.89314631</c:v>
+                  <c:v>2928125.55622932</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3110350.01450326</c:v>
+                  <c:v>3273525.21589428</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3427393.99548501</c:v>
+                  <c:v>3632626.9661002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3752096.55881845</c:v>
+                  <c:v>4006017.34994432</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4084377.48591498</c:v>
+                  <c:v>4394300.09637918</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4424112.64037826</c:v>
+                  <c:v>4798095.76601831</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4771128.501743</c:v>
+                  <c:v>5218041.26815356</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>5125196.16620118</c:v>
+                  <c:v>5654789.23282113</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5484617.52886721</c:v>
+                  <c:v>6107594.60599651</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5843082.11439971</c:v>
+                  <c:v>6571153.99449041</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6199266.7928546</c:v>
+                  <c:v>7045209.70059706</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>6551676.4122355</c:v>
+                  <c:v>7529415.05244095</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>6898626.69486865</c:v>
+                  <c:v>8023323.02868849</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>7238225.61039862</c:v>
+                  <c:v>8526373.700558</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7067914.70097689</c:v>
+                  <c:v>8535530.35606821</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>6853540.39329206</c:v>
+                  <c:v>8515793.26096971</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>6624590.64719421</c:v>
+                  <c:v>8497606.51093517</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6451880.56641936</c:v>
+                  <c:v>8552777.39560507</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6226408.78156159</c:v>
+                  <c:v>8573331.18392679</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1249,11 +1249,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="44370340"/>
-        <c:axId val="45776496"/>
+        <c:axId val="47628953"/>
+        <c:axId val="39150793"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="44370340"/>
+        <c:axId val="47628953"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1319,7 +1319,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45776496"/>
+        <c:crossAx val="39150793"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1327,7 +1327,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="45776496"/>
+        <c:axId val="39150793"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1403,7 +1403,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44370340"/>
+        <c:crossAx val="47628953"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1728,15 +1728,15 @@
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">INDEX(Model!$R$2:$R$27,15+1)</f>
-        <v>6582631.39844278</v>
+        <v>6582647.52498468</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">INDEX(Model!$R$2:$R$27,20+1)</f>
-        <v>10870780.1541459</v>
+        <v>10877297.8684327</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">INDEX(Model!$R$2:$R$27,25+1)</f>
-        <v>16940561.9261636</v>
+        <v>17042109.367774</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1745,27 +1745,27 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">INDEX(Model!$S$2:$S$27,1+1)</f>
-        <v>1105101.0744721</v>
+        <v>1112831.22078536</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">INDEX(Model!$S$2:$S$27,5+1)</f>
-        <v>2205414.37860174</v>
+        <v>2276173.60499552</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">INDEX(Model!$S$2:$S$27,10+1)</f>
-        <v>3752096.55881845</v>
+        <v>4006017.34994432</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">INDEX(Model!$S$2:$S$27,15+1)</f>
-        <v>5484617.52886721</v>
+        <v>6107594.60599651</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">INDEX(Model!$S$2:$S$27,20+1)</f>
-        <v>7238225.61039862</v>
+        <v>8526373.700558</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">INDEX(Model!$S$2:$S$27,25+1)</f>
-        <v>6226408.78156159</v>
+        <v>8573331.18392679</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,27 +1774,27 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">INDEX(Model!$T$2:$T$27,1+1)</f>
-        <v>-638854.401323989</v>
+        <v>-646584.547637244</v>
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">INDEX(Model!$T$2:$T$27,5+1)</f>
-        <v>-450285.038119031</v>
+        <v>-521044.264512806</v>
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">INDEX(Model!$T$2:$T$27,10+1)</f>
-        <v>145795.44507581</v>
+        <v>-108125.346050058</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">INDEX(Model!$T$2:$T$27,15+1)</f>
-        <v>1098013.86957557</v>
+        <v>475052.918988168</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">INDEX(Model!$T$2:$T$27,20+1)</f>
-        <v>3632554.54374725</v>
+        <v>2350924.16787468</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">INDEX(Model!$T$2:$T$27,25+1)</f>
-        <v>10714153.1446021</v>
+        <v>8468778.18384725</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1815,15 +1815,15 @@
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">INDEX(Model!$U$2:$U$27,15+1)</f>
-        <v>3401380.20780501</v>
+        <v>3401388.54071888</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">INDEX(Model!$U$2:$U$27,20+1)</f>
-        <v>4507491.37011747</v>
+        <v>4510193.89380796</v>
       </c>
       <c r="G8" s="6" t="n">
         <f aca="false">INDEX(Model!$U$2:$U$27,25+1)</f>
-        <v>5636643.27775186</v>
+        <v>5670431.21859001</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1832,27 +1832,27 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">INDEX(Model!$V$2:$V$27,1+1)</f>
-        <v>1057512.98992545</v>
+        <v>1064910.25912474</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">INDEX(Model!$V$2:$V$27,5+1)</f>
-        <v>1769737.07607662</v>
+        <v>1826517.89134589</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">INDEX(Model!$V$2:$V$27,10+1)</f>
-        <v>2416078.83987286</v>
+        <v>2579585.46632178</v>
       </c>
       <c r="E9" s="6" t="n">
         <f aca="false">INDEX(Model!$V$2:$V$27,15+1)</f>
-        <v>2834013.99544908</v>
+        <v>3155918.98629591</v>
       </c>
       <c r="F9" s="6" t="n">
         <f aca="false">INDEX(Model!$V$2:$V$27,20+1)</f>
-        <v>3001278.56613788</v>
+        <v>3535399.9739388</v>
       </c>
       <c r="G9" s="6" t="n">
         <f aca="false">INDEX(Model!$V$2:$V$27,25+1)</f>
-        <v>2071716.70904969</v>
+        <v>2852609.60034547</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">Inputs!$B$43</f>
-        <v>0.078</v>
+        <v>0.088</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Model!$A$3:$A$27,MATCH(TRUE(),INDEX(Model!$T$3:$T$27&gt;0,0),0)),"Not within 25y")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2281,7 +2281,7 @@
         <v>64</v>
       </c>
       <c r="B35" s="18" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="C35" s="14" t="s">
         <v>65</v>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="B43" s="20" t="n">
         <f aca="false">Inputs!$B$35-Inputs!$B$36-Inputs!$B$37-Inputs!$B$42</f>
-        <v>0.078</v>
+        <v>0.088</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>78</v>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="M3" s="16" t="n">
         <f aca="false">MAX(0,M2*(1+Inputs!$B$43)+L3*(1+Inputs!$B$43)^0.5)</f>
-        <v>1118364.57327809</v>
+        <v>1127791.58097718</v>
       </c>
       <c r="N3" s="16" t="n">
         <f aca="false">MAX(0,N2+L3)</f>
@@ -2730,11 +2730,11 @@
       </c>
       <c r="S3" s="24" t="n">
         <f aca="false">M3-MAX(0,M3-N3)*Inputs!$B$48</f>
-        <v>1105101.0744721</v>
+        <v>1112831.22078536</v>
       </c>
       <c r="T3" s="24" t="n">
         <f aca="false">R3-S3</f>
-        <v>-638854.401323989</v>
+        <v>-646584.547637244</v>
       </c>
       <c r="U3" s="16" t="n">
         <f aca="false">R3/(1+Inputs!$B$38)^A3</f>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="V3" s="16" t="n">
         <f aca="false">S3/(1+Inputs!$B$38)^A3</f>
-        <v>1057512.98992545</v>
+        <v>1064910.25912474</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="M4" s="16" t="n">
         <f aca="false">MAX(0,M3*(1+Inputs!$B$43)+L4*(1+Inputs!$B$43)^0.5)</f>
-        <v>1399289.20785801</v>
+        <v>1421625.75093545</v>
       </c>
       <c r="N4" s="16" t="n">
         <f aca="false">MAX(0,N3+L4)</f>
@@ -2819,11 +2819,11 @@
       </c>
       <c r="S4" s="24" t="n">
         <f aca="false">M4-MAX(0,M4-N4)*Inputs!$B$48</f>
-        <v>1369038.8542117</v>
+        <v>1387354.81953521</v>
       </c>
       <c r="T4" s="24" t="n">
         <f aca="false">R4-S4</f>
-        <v>-610256.819883226</v>
+        <v>-628572.785206729</v>
       </c>
       <c r="U4" s="16" t="n">
         <f aca="false">R4/(1+Inputs!$B$38)^A4</f>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="V4" s="16" t="n">
         <f aca="false">S4/(1+Inputs!$B$38)^A4</f>
-        <v>1253669.88320936</v>
+        <v>1270442.36124192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="M5" s="16" t="n">
         <f aca="false">MAX(0,M4*(1+Inputs!$B$43)+L5*(1+Inputs!$B$43)^0.5)</f>
-        <v>1691443.31751087</v>
+        <v>1730585.24735134</v>
       </c>
       <c r="N5" s="16" t="n">
         <f aca="false">MAX(0,N4+L5)</f>
@@ -2908,11 +2908,11 @@
       </c>
       <c r="S5" s="24" t="n">
         <f aca="false">M5-MAX(0,M5-N5)*Inputs!$B$48</f>
-        <v>1640332.79926112</v>
+        <v>1672429.1817303</v>
       </c>
       <c r="T5" s="24" t="n">
         <f aca="false">R5-S5</f>
-        <v>-570182.236493044</v>
+        <v>-602278.618962228</v>
       </c>
       <c r="U5" s="16" t="n">
         <f aca="false">R5/(1+Inputs!$B$38)^A5</f>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="V5" s="16" t="n">
         <f aca="false">S5/(1+Inputs!$B$38)^A5</f>
-        <v>1437418.0615124</v>
+        <v>1465544.0124726</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="M6" s="16" t="n">
         <f aca="false">MAX(0,M5*(1+Inputs!$B$43)+L6*(1+Inputs!$B$43)^0.5)</f>
-        <v>1995091.13840061</v>
+        <v>2055386.60558399</v>
       </c>
       <c r="N6" s="16" t="n">
         <f aca="false">MAX(0,N5+L6)</f>
@@ -2997,11 +2997,11 @@
       </c>
       <c r="S6" s="24" t="n">
         <f aca="false">M6-MAX(0,M6-N6)*Inputs!$B$48</f>
-        <v>1919093.54192227</v>
+        <v>1968535.82501265</v>
       </c>
       <c r="T6" s="24" t="n">
         <f aca="false">R6-S6</f>
-        <v>-517336.065386557</v>
+        <v>-566778.348476936</v>
       </c>
       <c r="U6" s="16" t="n">
         <f aca="false">R6/(1+Inputs!$B$38)^A6</f>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="V6" s="16" t="n">
         <f aca="false">S6/(1+Inputs!$B$38)^A6</f>
-        <v>1609277.6589954</v>
+        <v>1650738.04633399</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="M7" s="16" t="n">
         <f aca="false">MAX(0,M6*(1+Inputs!$B$43)+L7*(1+Inputs!$B$43)^0.5)</f>
-        <v>2310483.05201905</v>
+        <v>2396774.79152366</v>
       </c>
       <c r="N7" s="16" t="n">
         <f aca="false">MAX(0,N6+L7)</f>
@@ -3086,11 +3086,11 @@
       </c>
       <c r="S7" s="24" t="n">
         <f aca="false">M7-MAX(0,M7-N7)*Inputs!$B$48</f>
-        <v>2205414.37860174</v>
+        <v>2276173.60499552</v>
       </c>
       <c r="T7" s="24" t="n">
         <f aca="false">R7-S7</f>
-        <v>-450285.038119031</v>
+        <v>-521044.264512806</v>
       </c>
       <c r="U7" s="16" t="n">
         <f aca="false">R7/(1+Inputs!$B$38)^A7</f>
@@ -3098,7 +3098,7 @@
       </c>
       <c r="V7" s="16" t="n">
         <f aca="false">S7/(1+Inputs!$B$38)^A7</f>
-        <v>1769737.07607662</v>
+        <v>1826517.89134589</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="M8" s="16" t="n">
         <f aca="false">MAX(0,M7*(1+Inputs!$B$43)+L8*(1+Inputs!$B$43)^0.5)</f>
-        <v>2637852.60224202</v>
+        <v>2755523.79239606</v>
       </c>
       <c r="N8" s="16" t="n">
         <f aca="false">MAX(0,N7+L8)</f>
@@ -3175,11 +3175,11 @@
       </c>
       <c r="S8" s="24" t="n">
         <f aca="false">M8-MAX(0,M8-N8)*Inputs!$B$48</f>
-        <v>2499368.49400676</v>
+        <v>2595858.86993307</v>
       </c>
       <c r="T8" s="24" t="n">
         <f aca="false">R8-S8</f>
-        <v>-367442.730584596</v>
+        <v>-463933.106510911</v>
       </c>
       <c r="U8" s="16" t="n">
         <f aca="false">R8/(1+Inputs!$B$38)^A8</f>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="V8" s="16" t="n">
         <f aca="false">S8/(1+Inputs!$B$38)^A8</f>
-        <v>1919254.41493451</v>
+        <v>1993348.96339318</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="M9" s="16" t="n">
         <f aca="false">MAX(0,M8*(1+Inputs!$B$43)+L9*(1+Inputs!$B$43)^0.5)</f>
-        <v>2977413.17763266</v>
+        <v>3132437.15700219</v>
       </c>
       <c r="N9" s="16" t="n">
         <f aca="false">MAX(0,N8+L9)</f>
@@ -3264,11 +3264,11 @@
       </c>
       <c r="S9" s="24" t="n">
         <f aca="false">M9-MAX(0,M9-N9)*Inputs!$B$48</f>
-        <v>2801005.89314631</v>
+        <v>2928125.55622932</v>
       </c>
       <c r="T9" s="24" t="n">
         <f aca="false">R9-S9</f>
-        <v>-267053.592551312</v>
+        <v>-394173.255634323</v>
       </c>
       <c r="U9" s="16" t="n">
         <f aca="false">R9/(1+Inputs!$B$38)^A9</f>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="V9" s="16" t="n">
         <f aca="false">S9/(1+Inputs!$B$38)^A9</f>
-        <v>2058258.84042017</v>
+        <v>2151669.98638457</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="M10" s="16" t="n">
         <f aca="false">MAX(0,M9*(1+Inputs!$B$43)+L10*(1+Inputs!$B$43)^0.5)</f>
-        <v>3329354.32762334</v>
+        <v>3528348.47566117</v>
       </c>
       <c r="N10" s="16" t="n">
         <f aca="false">MAX(0,N9+L10)</f>
@@ -3353,11 +3353,11 @@
       </c>
       <c r="S10" s="24" t="n">
         <f aca="false">M10-MAX(0,M10-N10)*Inputs!$B$48</f>
-        <v>3110350.01450326</v>
+        <v>3273525.21589428</v>
       </c>
       <c r="T10" s="24" t="n">
         <f aca="false">R10-S10</f>
-        <v>-147175.32444285</v>
+        <v>-310350.525833869</v>
       </c>
       <c r="U10" s="16" t="n">
         <f aca="false">R10/(1+Inputs!$B$38)^A10</f>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="V10" s="16" t="n">
         <f aca="false">S10/(1+Inputs!$B$38)^A10</f>
-        <v>2187151.86986606</v>
+        <v>2301894.24457437</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="M11" s="16" t="n">
         <f aca="false">MAX(0,M10*(1+Inputs!$B$43)+L11*(1+Inputs!$B$43)^0.5)</f>
-        <v>3693837.6785064</v>
+        <v>3944121.78901273</v>
       </c>
       <c r="N11" s="16" t="n">
         <f aca="false">MAX(0,N10+L11)</f>
@@ -3442,11 +3442,11 @@
       </c>
       <c r="S11" s="24" t="n">
         <f aca="false">M11-MAX(0,M11-N11)*Inputs!$B$48</f>
-        <v>3427393.99548501</v>
+        <v>3632626.9661002</v>
       </c>
       <c r="T11" s="24" t="n">
         <f aca="false">R11-S11</f>
-        <v>-5659.42986985529</v>
+        <v>-210892.400485044</v>
       </c>
       <c r="U11" s="16" t="n">
         <f aca="false">R11/(1+Inputs!$B$38)^A11</f>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="V11" s="16" t="n">
         <f aca="false">S11/(1+Inputs!$B$38)^A11</f>
-        <v>2306308.59510759</v>
+        <v>2444410.76974896</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="M12" s="16" t="n">
         <f aca="false">MAX(0,M11*(1+Inputs!$B$43)+L12*(1+Inputs!$B$43)^0.5)</f>
-        <v>4070992.41224282</v>
+        <v>4380651.91361583</v>
       </c>
       <c r="N12" s="16" t="n">
         <f aca="false">MAX(0,N11+L12)</f>
@@ -3531,11 +3531,11 @@
       </c>
       <c r="S12" s="24" t="n">
         <f aca="false">M12-MAX(0,M12-N12)*Inputs!$B$48</f>
-        <v>3752096.55881845</v>
+        <v>4006017.34994432</v>
       </c>
       <c r="T12" s="24" t="n">
         <f aca="false">R12-S12</f>
-        <v>145795.44507581</v>
+        <v>-108125.346050058</v>
       </c>
       <c r="U12" s="16" t="n">
         <f aca="false">R12/(1+Inputs!$B$38)^A12</f>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="V12" s="16" t="n">
         <f aca="false">S12/(1+Inputs!$B$38)^A12</f>
-        <v>2416078.83987286</v>
+        <v>2579585.46632178</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="M13" s="16" t="n">
         <f aca="false">MAX(0,M12*(1+Inputs!$B$43)+L13*(1+Inputs!$B$43)^0.5)</f>
-        <v>4460910.2679362</v>
+        <v>4838864.67094131</v>
       </c>
       <c r="N13" s="16" t="n">
         <f aca="false">MAX(0,N12+L13)</f>
@@ -3620,11 +3620,11 @@
       </c>
       <c r="S13" s="24" t="n">
         <f aca="false">M13-MAX(0,M13-N13)*Inputs!$B$48</f>
-        <v>4084377.48591498</v>
+        <v>4394300.09637918</v>
       </c>
       <c r="T13" s="24" t="n">
         <f aca="false">R13-S13</f>
-        <v>275789.453693348</v>
+        <v>-34133.156770844</v>
       </c>
       <c r="U13" s="16" t="n">
         <f aca="false">R13/(1+Inputs!$B$38)^A13</f>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="V13" s="16" t="n">
         <f aca="false">S13/(1+Inputs!$B$38)^A13</f>
-        <v>2516788.25554156</v>
+        <v>2707762.17723047</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="M14" s="16" t="n">
         <f aca="false">MAX(0,M13*(1+Inputs!$B$43)+L14*(1+Inputs!$B$43)^0.5)</f>
-        <v>4863640.02240086</v>
+        <v>5319717.00488872</v>
       </c>
       <c r="N14" s="16" t="n">
         <f aca="false">MAX(0,N13+L14)</f>
@@ -3709,11 +3709,11 @@
       </c>
       <c r="S14" s="24" t="n">
         <f aca="false">M14-MAX(0,M14-N14)*Inputs!$B$48</f>
-        <v>4424112.64037826</v>
+        <v>4798095.76601831</v>
       </c>
       <c r="T14" s="24" t="n">
         <f aca="false">R14-S14</f>
-        <v>432220.86910428</v>
+        <v>58237.7434642315</v>
       </c>
       <c r="U14" s="16" t="n">
         <f aca="false">R14/(1+Inputs!$B$38)^A14</f>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="V14" s="16" t="n">
         <f aca="false">S14/(1+Inputs!$B$38)^A14</f>
-        <v>2608739.35812695</v>
+        <v>2829263.69338644</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="M15" s="16" t="n">
         <f aca="false">MAX(0,M14*(1+Inputs!$B$43)+L15*(1+Inputs!$B$43)^0.5)</f>
-        <v>5279181.40255507</v>
+        <v>5824196.97134843</v>
       </c>
       <c r="N15" s="16" t="n">
         <f aca="false">MAX(0,N14+L15)</f>
@@ -3798,11 +3798,11 @@
       </c>
       <c r="S15" s="24" t="n">
         <f aca="false">M15-MAX(0,M15-N15)*Inputs!$B$48</f>
-        <v>4771128.501743</v>
+        <v>5218041.26815356</v>
       </c>
       <c r="T15" s="24" t="n">
         <f aca="false">R15-S15</f>
-        <v>618145.553859124</v>
+        <v>171232.787448567</v>
       </c>
       <c r="U15" s="16" t="n">
         <f aca="false">R15/(1+Inputs!$B$38)^A15</f>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="V15" s="16" t="n">
         <f aca="false">S15/(1+Inputs!$B$38)^A15</f>
-        <v>2692212.50919523</v>
+        <v>2944392.70929044</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="M16" s="16" t="n">
         <f aca="false">MAX(0,M15*(1+Inputs!$B$43)+L16*(1+Inputs!$B$43)^0.5)</f>
-        <v>5707478.3783721</v>
+        <v>6353323.58156717</v>
       </c>
       <c r="N16" s="16" t="n">
         <f aca="false">MAX(0,N15+L16)</f>
@@ -3887,11 +3887,11 @@
       </c>
       <c r="S16" s="24" t="n">
         <f aca="false">M16-MAX(0,M16-N16)*Inputs!$B$48</f>
-        <v>5125196.16620118</v>
+        <v>5654789.23282113</v>
       </c>
       <c r="T16" s="24" t="n">
         <f aca="false">R16-S16</f>
-        <v>836949.766247312</v>
+        <v>307356.699627358</v>
       </c>
       <c r="U16" s="16" t="n">
         <f aca="false">R16/(1+Inputs!$B$38)^A16</f>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="V16" s="16" t="n">
         <f aca="false">S16/(1+Inputs!$B$38)^A16</f>
-        <v>2767466.8433025</v>
+        <v>3053432.72729714</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="M17" s="16" t="n">
         <f aca="false">MAX(0,M16*(1+Inputs!$B$43)+L17*(1+Inputs!$B$43)^0.5)</f>
-        <v>6146995.14377086</v>
+        <v>6906723.28661147</v>
       </c>
       <c r="N17" s="16" t="n">
         <f aca="false">MAX(0,N16+L17)</f>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="P17" s="16" t="n">
         <f aca="false">P16*(1+Inputs!$B$43)+O17*(1+Inputs!$B$43)^0.5</f>
-        <v>4249.9110856959</v>
+        <v>4269.57760020276</v>
       </c>
       <c r="Q17" s="16" t="n">
         <f aca="false">Q16+O17</f>
@@ -3972,23 +3972,23 @@
       </c>
       <c r="R17" s="24" t="n">
         <f aca="false">B17*(1-Inputs!$B$46)-C17-MAX(0,B17*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P17-MAX(0,P17-Q17)*Inputs!$B$48</f>
-        <v>6582631.39844278</v>
+        <v>6582647.52498468</v>
       </c>
       <c r="S17" s="24" t="n">
         <f aca="false">M17-MAX(0,M17-N17)*Inputs!$B$48</f>
-        <v>5484617.52886721</v>
+        <v>6107594.60599651</v>
       </c>
       <c r="T17" s="24" t="n">
         <f aca="false">R17-S17</f>
-        <v>1098013.86957557</v>
+        <v>475052.918988168</v>
       </c>
       <c r="U17" s="16" t="n">
         <f aca="false">R17/(1+Inputs!$B$38)^A17</f>
-        <v>3401380.20780501</v>
+        <v>3401388.54071888</v>
       </c>
       <c r="V17" s="16" t="n">
         <f aca="false">S17/(1+Inputs!$B$38)^A17</f>
-        <v>2834013.99544908</v>
+        <v>3155918.98629591</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="M18" s="16" t="n">
         <f aca="false">MAX(0,M17*(1+Inputs!$B$43)+L18*(1+Inputs!$B$43)^0.5)</f>
-        <v>6591531.81122767</v>
+        <v>7479424.34792364</v>
       </c>
       <c r="N18" s="16" t="n">
         <f aca="false">MAX(0,N17+L18)</f>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="P18" s="16" t="n">
         <f aca="false">P17*(1+Inputs!$B$43)+O18*(1+Inputs!$B$43)^0.5</f>
-        <v>30778.1194683731</v>
+        <v>30963.2413612546</v>
       </c>
       <c r="Q18" s="16" t="n">
         <f aca="false">Q17+O18</f>
@@ -4061,23 +4061,23 @@
       </c>
       <c r="R18" s="24" t="n">
         <f aca="false">B18*(1-Inputs!$B$46)-C18-MAX(0,B18*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P18-MAX(0,P18-Q18)*Inputs!$B$48</f>
-        <v>7272376.66912875</v>
+        <v>7272528.46908091</v>
       </c>
       <c r="S18" s="24" t="n">
         <f aca="false">M18-MAX(0,M18-N18)*Inputs!$B$48</f>
-        <v>5843082.11439971</v>
+        <v>6571153.99449041</v>
       </c>
       <c r="T18" s="24" t="n">
         <f aca="false">R18-S18</f>
-        <v>1429294.55472903</v>
+        <v>701374.474590498</v>
       </c>
       <c r="U18" s="16" t="n">
         <f aca="false">R18/(1+Inputs!$B$38)^A18</f>
-        <v>3595967.1666594</v>
+        <v>3596042.22707895</v>
       </c>
       <c r="V18" s="16" t="n">
         <f aca="false">S18/(1+Inputs!$B$38)^A18</f>
-        <v>2889224.8561148</v>
+        <v>3249234.06560585</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="M19" s="16" t="n">
         <f aca="false">MAX(0,M18*(1+Inputs!$B$43)+L19*(1+Inputs!$B$43)^0.5)</f>
-        <v>7039824.74920187</v>
+        <v>8071462.44157071</v>
       </c>
       <c r="N19" s="16" t="n">
         <f aca="false">MAX(0,N18+L19)</f>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="P19" s="16" t="n">
         <f aca="false">P18*(1+Inputs!$B$43)+O19*(1+Inputs!$B$43)^0.5</f>
-        <v>82563.7202630758</v>
+        <v>83301.4433287016</v>
       </c>
       <c r="Q19" s="16" t="n">
         <f aca="false">Q18+O19</f>
@@ -4150,23 +4150,23 @@
       </c>
       <c r="R19" s="24" t="n">
         <f aca="false">B19*(1-Inputs!$B$46)-C19-MAX(0,B19*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P19-MAX(0,P19-Q19)*Inputs!$B$48</f>
-        <v>8038203.58167651</v>
+        <v>8038808.51459033</v>
       </c>
       <c r="S19" s="24" t="n">
         <f aca="false">M19-MAX(0,M19-N19)*Inputs!$B$48</f>
-        <v>6199266.7928546</v>
+        <v>7045209.70059706</v>
       </c>
       <c r="T19" s="24" t="n">
         <f aca="false">R19-S19</f>
-        <v>1838936.78882191</v>
+        <v>993598.813993269</v>
       </c>
       <c r="U19" s="16" t="n">
         <f aca="false">R19/(1+Inputs!$B$38)^A19</f>
-        <v>3803488.11625016</v>
+        <v>3803774.35621975</v>
       </c>
       <c r="V19" s="16" t="n">
         <f aca="false">S19/(1+Inputs!$B$38)^A19</f>
-        <v>2933346.65345325</v>
+        <v>3333626.8608318</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="M20" s="16" t="n">
         <f aca="false">MAX(0,M19*(1+Inputs!$B$43)+L20*(1+Inputs!$B$43)^0.5)</f>
-        <v>7490419.95362151</v>
+        <v>8682784.14899401</v>
       </c>
       <c r="N20" s="16" t="n">
         <f aca="false">MAX(0,N19+L20)</f>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="P20" s="16" t="n">
         <f aca="false">P19*(1+Inputs!$B$43)+O20*(1+Inputs!$B$43)^0.5</f>
-        <v>162887.03495717</v>
+        <v>164857.210917823</v>
       </c>
       <c r="Q20" s="16" t="n">
         <f aca="false">Q19+O20</f>
@@ -4239,23 +4239,23 @@
       </c>
       <c r="R20" s="24" t="n">
         <f aca="false">B20*(1-Inputs!$B$46)-C20-MAX(0,B20*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P20-MAX(0,P20-Q20)*Inputs!$B$48</f>
-        <v>8887599.9585631</v>
+        <v>8889215.50285084</v>
       </c>
       <c r="S20" s="24" t="n">
         <f aca="false">M20-MAX(0,M20-N20)*Inputs!$B$48</f>
-        <v>6551676.4122355</v>
+        <v>7529415.05244095</v>
       </c>
       <c r="T20" s="24" t="n">
         <f aca="false">R20-S20</f>
-        <v>2335923.5463276</v>
+        <v>1359800.45040989</v>
       </c>
       <c r="U20" s="16" t="n">
         <f aca="false">R20/(1+Inputs!$B$38)^A20</f>
-        <v>4024308.53940247</v>
+        <v>4025040.05845184</v>
       </c>
       <c r="V20" s="16" t="n">
         <f aca="false">S20/(1+Inputs!$B$38)^A20</f>
-        <v>2966601.4960268</v>
+        <v>3409321.91294785</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="M21" s="16" t="n">
         <f aca="false">MAX(0,M20*(1+Inputs!$B$43)+L21*(1+Inputs!$B$43)^0.5)</f>
-        <v>7941653.23851967</v>
+        <v>9313234.13342192</v>
       </c>
       <c r="N21" s="16" t="n">
         <f aca="false">MAX(0,N20+L21)</f>
@@ -4320,7 +4320,7 @@
       </c>
       <c r="P21" s="16" t="n">
         <f aca="false">P20*(1+Inputs!$B$43)+O21*(1+Inputs!$B$43)^0.5</f>
-        <v>275356.827297067</v>
+        <v>279590.91099126</v>
       </c>
       <c r="Q21" s="16" t="n">
         <f aca="false">Q20+O21</f>
@@ -4328,23 +4328,23 @@
       </c>
       <c r="R21" s="24" t="n">
         <f aca="false">B21*(1-Inputs!$B$46)-C21-MAX(0,B21*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P21-MAX(0,P21-Q21)*Inputs!$B$48</f>
-        <v>9828784.8360684</v>
+        <v>9832256.78469764</v>
       </c>
       <c r="S21" s="24" t="n">
         <f aca="false">M21-MAX(0,M21-N21)*Inputs!$B$48</f>
-        <v>6898626.69486865</v>
+        <v>8023323.02868849</v>
       </c>
       <c r="T21" s="24" t="n">
         <f aca="false">R21-S21</f>
-        <v>2930158.14119975</v>
+        <v>1808933.75600915</v>
       </c>
       <c r="U21" s="16" t="n">
         <f aca="false">R21/(1+Inputs!$B$38)^A21</f>
-        <v>4258830.04697621</v>
+        <v>4260334.44852639</v>
       </c>
       <c r="V21" s="16" t="n">
         <f aca="false">S21/(1+Inputs!$B$38)^A21</f>
-        <v>2989187.2841863</v>
+        <v>3476520.21700406</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="M22" s="16" t="n">
         <f aca="false">MAX(0,M21*(1+Inputs!$B$43)+L22*(1+Inputs!$B$43)^0.5)</f>
-        <v>8391628.62345583</v>
+        <v>9962540.92852824</v>
       </c>
       <c r="N22" s="16" t="n">
         <f aca="false">MAX(0,N21+L22)</f>
@@ -4409,7 +4409,7 @@
       </c>
       <c r="P22" s="16" t="n">
         <f aca="false">P21*(1+Inputs!$B$43)+O22*(1+Inputs!$B$43)^0.5</f>
-        <v>423939.835577526</v>
+        <v>431888.267634599</v>
       </c>
       <c r="Q22" s="16" t="n">
         <f aca="false">Q21+O22</f>
@@ -4417,23 +4417,23 @@
       </c>
       <c r="R22" s="24" t="n">
         <f aca="false">B22*(1-Inputs!$B$46)-C22-MAX(0,B22*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P22-MAX(0,P22-Q22)*Inputs!$B$48</f>
-        <v>10870780.1541459</v>
+        <v>10877297.8684327</v>
       </c>
       <c r="S22" s="24" t="n">
         <f aca="false">M22-MAX(0,M22-N22)*Inputs!$B$48</f>
-        <v>7238225.61039862</v>
+        <v>8526373.700558</v>
       </c>
       <c r="T22" s="24" t="n">
         <f aca="false">R22-S22</f>
-        <v>3632554.54374725</v>
+        <v>2350924.16787468</v>
       </c>
       <c r="U22" s="16" t="n">
         <f aca="false">R22/(1+Inputs!$B$38)^A22</f>
-        <v>4507491.37011747</v>
+        <v>4510193.89380796</v>
       </c>
       <c r="V22" s="16" t="n">
         <f aca="false">S22/(1+Inputs!$B$38)^A22</f>
-        <v>3001278.56613788</v>
+        <v>3535399.9739388</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="M23" s="16" t="n">
         <f aca="false">MAX(0,M22*(1+Inputs!$B$43)+L23*(1+Inputs!$B$43)^0.5)</f>
-        <v>8334414.1253797</v>
+        <v>10124189.3145154</v>
       </c>
       <c r="N23" s="16" t="n">
         <f aca="false">MAX(0,N22+L23)</f>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="P23" s="16" t="n">
         <f aca="false">P22*(1+Inputs!$B$43)+O23*(1+Inputs!$B$43)^0.5</f>
-        <v>990828.290781837</v>
+        <v>1006185.8469789</v>
       </c>
       <c r="Q23" s="16" t="n">
         <f aca="false">Q22+O23</f>
@@ -4506,23 +4506,23 @@
       </c>
       <c r="R23" s="24" t="n">
         <f aca="false">B23*(1-Inputs!$B$46)-C23-MAX(0,B23*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P23-MAX(0,P23-Q23)*Inputs!$B$48</f>
-        <v>11889560.2077326</v>
+        <v>11902153.4038142</v>
       </c>
       <c r="S23" s="24" t="n">
         <f aca="false">M23-MAX(0,M23-N23)*Inputs!$B$48</f>
-        <v>7067914.70097689</v>
+        <v>8535530.35606821</v>
       </c>
       <c r="T23" s="24" t="n">
         <f aca="false">R23-S23</f>
-        <v>4821645.50675569</v>
+        <v>3366623.04774597</v>
       </c>
       <c r="U23" s="16" t="n">
         <f aca="false">R23/(1+Inputs!$B$38)^A23</f>
-        <v>4717627.98557538</v>
+        <v>4722624.80742786</v>
       </c>
       <c r="V23" s="16" t="n">
         <f aca="false">S23/(1+Inputs!$B$38)^A23</f>
-        <v>2804459.67810504</v>
+        <v>3386791.11556431</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M24" s="16" t="n">
         <f aca="false">MAX(0,M23*(1+Inputs!$B$43)+L24*(1+Inputs!$B$43)^0.5)</f>
-        <v>8232063.09442524</v>
+        <v>10259200.7379346</v>
       </c>
       <c r="N24" s="16" t="n">
         <f aca="false">MAX(0,N23+L24)</f>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="P24" s="16" t="n">
         <f aca="false">P23*(1+Inputs!$B$43)+O24*(1+Inputs!$B$43)^0.5</f>
-        <v>1632439.39701337</v>
+        <v>1661668.12870673</v>
       </c>
       <c r="Q24" s="16" t="n">
         <f aca="false">Q23+O24</f>
@@ -4595,23 +4595,23 @@
       </c>
       <c r="R24" s="24" t="n">
         <f aca="false">B24*(1-Inputs!$B$46)-C24-MAX(0,B24*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P24-MAX(0,P24-Q24)*Inputs!$B$48</f>
-        <v>12997970.6788673</v>
+        <v>13021938.2388558</v>
       </c>
       <c r="S24" s="24" t="n">
         <f aca="false">M24-MAX(0,M24-N24)*Inputs!$B$48</f>
-        <v>6853540.39329206</v>
+        <v>8515793.26096971</v>
       </c>
       <c r="T24" s="24" t="n">
         <f aca="false">R24-S24</f>
-        <v>6144430.28557519</v>
+        <v>4506144.9778861</v>
       </c>
       <c r="U24" s="16" t="n">
         <f aca="false">R24/(1+Inputs!$B$38)^A24</f>
-        <v>4935340.97880717</v>
+        <v>4944441.4825624</v>
       </c>
       <c r="V24" s="16" t="n">
         <f aca="false">S24/(1+Inputs!$B$38)^A24</f>
-        <v>2602295.35737591</v>
+        <v>3233454.24345705</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="M25" s="16" t="n">
         <f aca="false">MAX(0,M24*(1+Inputs!$B$43)+L25*(1+Inputs!$B$43)^0.5)</f>
-        <v>8078769.08194415</v>
+        <v>10362934.7694331</v>
       </c>
       <c r="N25" s="16" t="n">
         <f aca="false">MAX(0,N24+L25)</f>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="P25" s="16" t="n">
         <f aca="false">P24*(1+Inputs!$B$43)+O25*(1+Inputs!$B$43)^0.5</f>
-        <v>2356315.87036511</v>
+        <v>2407201.64911267</v>
       </c>
       <c r="Q25" s="16" t="n">
         <f aca="false">Q24+O25</f>
@@ -4684,23 +4684,23 @@
       </c>
       <c r="R25" s="24" t="n">
         <f aca="false">B25*(1-Inputs!$B$46)-C25-MAX(0,B25*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P25-MAX(0,P25-Q25)*Inputs!$B$48</f>
-        <v>14203647.2672151</v>
+        <v>14245373.6057881</v>
       </c>
       <c r="S25" s="24" t="n">
         <f aca="false">M25-MAX(0,M25-N25)*Inputs!$B$48</f>
-        <v>6624590.64719421</v>
+        <v>8497606.51093517</v>
       </c>
       <c r="T25" s="24" t="n">
         <f aca="false">R25-S25</f>
-        <v>7579056.62002088</v>
+        <v>5747767.09485292</v>
       </c>
       <c r="U25" s="16" t="n">
         <f aca="false">R25/(1+Inputs!$B$38)^A25</f>
-        <v>5160897.07870464</v>
+        <v>5176058.34924277</v>
       </c>
       <c r="V25" s="16" t="n">
         <f aca="false">S25/(1+Inputs!$B$38)^A25</f>
-        <v>2407045.87177643</v>
+        <v>3087606.42905388</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="M26" s="16" t="n">
         <f aca="false">MAX(0,M25*(1+Inputs!$B$43)+L26*(1+Inputs!$B$43)^0.5)</f>
-        <v>7868147.03221873</v>
+        <v>10430216.3361037</v>
       </c>
       <c r="N26" s="16" t="n">
         <f aca="false">MAX(0,N25+L26)</f>
@@ -4765,7 +4765,7 @@
       </c>
       <c r="P26" s="16" t="n">
         <f aca="false">P25*(1+Inputs!$B$43)+O26*(1+Inputs!$B$43)^0.5</f>
-        <v>3170683.03684139</v>
+        <v>3252527.91401422</v>
       </c>
       <c r="Q26" s="16" t="n">
         <f aca="false">Q25+O26</f>
@@ -4773,23 +4773,23 @@
       </c>
       <c r="R26" s="24" t="n">
         <f aca="false">B26*(1-Inputs!$B$46)-C26-MAX(0,B26*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P26-MAX(0,P26-Q26)*Inputs!$B$48</f>
-        <v>15514859.4303046</v>
+        <v>15581972.2295863</v>
       </c>
       <c r="S26" s="24" t="n">
         <f aca="false">M26-MAX(0,M26-N26)*Inputs!$B$48</f>
-        <v>6451880.56641936</v>
+        <v>8552777.39560507</v>
       </c>
       <c r="T26" s="24" t="n">
         <f aca="false">R26-S26</f>
-        <v>9062978.86388524</v>
+        <v>7029194.83398126</v>
       </c>
       <c r="U26" s="16" t="n">
         <f aca="false">R26/(1+Inputs!$B$38)^A26</f>
-        <v>5394570.51522235</v>
+        <v>5417905.86865082</v>
       </c>
       <c r="V26" s="16" t="n">
         <f aca="false">S26/(1+Inputs!$B$38)^A26</f>
-        <v>2243341.28373464</v>
+        <v>2973830.40876739</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="M27" s="16" t="n">
         <f aca="false">MAX(0,M26*(1+Inputs!$B$43)+L27*(1+Inputs!$B$43)^0.5)</f>
-        <v>7593181.44092876</v>
+        <v>10455281.931618</v>
       </c>
       <c r="N27" s="16" t="n">
         <f aca="false">MAX(0,N26+L27)</f>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="P27" s="16" t="n">
         <f aca="false">P26*(1+Inputs!$B$43)+O27*(1+Inputs!$B$43)^0.5</f>
-        <v>4084507.10856729</v>
+        <v>4208345.4519946</v>
       </c>
       <c r="Q27" s="16" t="n">
         <f aca="false">Q26+O27</f>
@@ -4862,23 +4862,23 @@
       </c>
       <c r="R27" s="24" t="n">
         <f aca="false">B27*(1-Inputs!$B$46)-C27-MAX(0,B27*(1-Inputs!$B$46)-(Inputs!$B$6+Inputs!$B$10+Inputs!$B$11)-Inputs!$B$47)*Inputs!$B$48+P27-MAX(0,P27-Q27)*Inputs!$B$48</f>
-        <v>16940561.9261636</v>
+        <v>17042109.367774</v>
       </c>
       <c r="S27" s="24" t="n">
         <f aca="false">M27-MAX(0,M27-N27)*Inputs!$B$48</f>
-        <v>6226408.78156159</v>
+        <v>8573331.18392679</v>
       </c>
       <c r="T27" s="24" t="n">
         <f aca="false">R27-S27</f>
-        <v>10714153.1446021</v>
+        <v>8468778.18384725</v>
       </c>
       <c r="U27" s="16" t="n">
         <f aca="false">R27/(1+Inputs!$B$38)^A27</f>
-        <v>5636643.27775186</v>
+        <v>5670431.21859001</v>
       </c>
       <c r="V27" s="16" t="n">
         <f aca="false">S27/(1+Inputs!$B$38)^A27</f>
-        <v>2071716.70904969</v>
+        <v>2852609.60034547</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>